<commit_message>
투자 대시보드 2026-10-15 18:25
</commit_message>
<xml_diff>
--- a/technicals/exports/2026-10-14.xlsx
+++ b/technicals/exports/2026-10-14.xlsx
@@ -122,55 +122,55 @@
       </ns0:c>
       <ns0:c r="B2" t="inlineStr">
         <ns0:is>
-          <ns0:t>ATKR</ns0:t>
+          <ns0:t>ABBV</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="C2" t="inlineStr">
         <ns0:is>
-          <ns0:t>Atkore Inc</ns0:t>
+          <ns0:t>Abbvie Inc</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D2" t="inlineStr">
         <ns0:is>
-          <ns0:t>Industrials</ns0:t>
+          <ns0:t>Healthcare</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="E2" t="inlineStr">
         <ns0:is>
-          <ns0:t>Electrical Equipment &amp; Parts</ns0:t>
+          <ns0:t>Drug Manufacturers - General</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F2" t="inlineStr">
         <ns0:is>
-          <ns0:t>전기·기계·안전·인프라 제품과 솔루션을 제조·판매하는 기업.</ns0:t>
+          <ns0:t>전 세계에서 의약품·치료제를 연구·개발·제조·판매하는 연구 중심 바이오 제약 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G2">
-        <ns0:v>94.93000030517578</ns0:v>
+        <ns0:v>283.4800109863281</ns0:v>
       </ns0:c>
       <ns0:c r="H2">
-        <ns0:v>0.052701362990403844</ns0:v>
+        <ns0:v>3.3241092439479925</ns0:v>
       </ns0:c>
       <ns0:c r="I2">
-        <ns0:v>94.9000015258789</ns0:v>
+        <ns0:v>283.42999267578125</ns0:v>
       </ns0:c>
       <ns0:c r="J2">
-        <ns0:v>0.0316109365801065</ns0:v>
+        <ns0:v>0.017647500913597902</ns0:v>
       </ns0:c>
       <ns0:c r="K2">
-        <ns0:v>1.149775972643658</ns0:v>
+        <ns0:v>1.201887444117473</ns0:v>
       </ns0:c>
       <ns0:c r="L2">
-        <ns0:v>72.23885089238354</ns0:v>
+        <ns0:v>69.68325183031487</ns0:v>
       </ns0:c>
       <ns0:c r="M2">
-        <ns0:v>94.67849960327149</ns0:v>
+        <ns0:v>267.8889984130859</ns0:v>
       </ns0:c>
       <ns0:c r="N2">
-        <ns0:v>94.14320022583007</ns0:v>
+        <ns0:v>260.8753985595703</ns0:v>
       </ns0:c>
       <ns0:c r="O2">
-        <ns0:v>76.60020009994507</ns0:v>
+        <ns0:v>233.40449935913085</ns0:v>
       </ns0:c>
       <ns0:c r="P2" t="inlineStr">
         <ns0:is>
@@ -189,7 +189,7 @@
       </ns0:c>
       <ns0:c r="T2" t="inlineStr">
         <ns0:is>
-          <ns0:t>https://finance.yahoo.com/quote/ATKR/profile/</ns0:t>
+          <ns0:t>https://finance.yahoo.com/quote/ABBV/profile/</ns0:t>
         </ns0:is>
       </ns0:c>
     </ns0:row>
@@ -201,55 +201,52 @@
       </ns0:c>
       <ns0:c r="B3" t="inlineStr">
         <ns0:is>
-          <ns0:t>ABBV</ns0:t>
+          <ns0:t>ALDF</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="C3" t="inlineStr">
         <ns0:is>
-          <ns0:t>Abbvie Inc</ns0:t>
+          <ns0:t>Aldel Financial II Inc</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D3" t="inlineStr">
         <ns0:is>
-          <ns0:t>Healthcare</ns0:t>
+          <ns0:t>Financial</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="E3" t="inlineStr">
         <ns0:is>
-          <ns0:t>Drug Manufacturers - General</ns0:t>
+          <ns0:t>Shell Companies</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F3" t="inlineStr">
         <ns0:is>
-          <ns0:t>전 세계에서 의약품과 치료제를 연구·개발·제조·판매하는 연구 중심 바이오 제약 기업.</ns0:t>
+          <ns0:t>주요 영업활동 없이 합병·주식교환·자산인수 등 사업결합을 추진하는 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G3">
-        <ns0:v>283.4800109863281</ns0:v>
+        <ns0:v>10.979999542236328</ns0:v>
       </ns0:c>
       <ns0:c r="H3">
-        <ns0:v>3.3241092439479925</ns0:v>
+        <ns0:v>1.4787416998601755</ns0:v>
       </ns0:c>
       <ns0:c r="I3">
-        <ns0:v>283.42999267578125</ns0:v>
+        <ns0:v>10.859999656677246</ns0:v>
       </ns0:c>
       <ns0:c r="J3">
-        <ns0:v>0.017647500913597902</ns0:v>
-      </ns0:c>
-      <ns0:c r="K3">
-        <ns0:v>1.201887444117473</ns0:v>
+        <ns0:v>1.1049713568388686</ns0:v>
       </ns0:c>
       <ns0:c r="L3">
-        <ns0:v>69.68325183031487</ns0:v>
+        <ns0:v>94.11871785465019</ns0:v>
       </ns0:c>
       <ns0:c r="M3">
-        <ns0:v>267.8889984130859</ns0:v>
+        <ns0:v>10.829999732971192</ns0:v>
       </ns0:c>
       <ns0:c r="N3">
-        <ns0:v>260.8753985595703</ns0:v>
+        <ns0:v>10.801599884033203</ns0:v>
       </ns0:c>
       <ns0:c r="O3">
-        <ns0:v>233.40449935913085</ns0:v>
+        <ns0:v>10.65395495414734</ns0:v>
       </ns0:c>
       <ns0:c r="P3" t="inlineStr">
         <ns0:is>
@@ -268,7 +265,7 @@
       </ns0:c>
       <ns0:c r="T3" t="inlineStr">
         <ns0:is>
-          <ns0:t>https://finance.yahoo.com/quote/ABBV/profile/</ns0:t>
+          <ns0:t>https://finance.yahoo.com/quote/ALDF/profile/</ns0:t>
         </ns0:is>
       </ns0:c>
     </ns0:row>
@@ -280,56 +277,59 @@
       </ns0:c>
       <ns0:c r="B4" t="inlineStr">
         <ns0:is>
-          <ns0:t>ALDF</ns0:t>
+          <ns0:t>APA</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="C4" t="inlineStr">
         <ns0:is>
-          <ns0:t>Aldel Financial II Inc</ns0:t>
+          <ns0:t>APA Corp</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D4" t="inlineStr">
         <ns0:is>
-          <ns0:t>Financial</ns0:t>
+          <ns0:t>Energy</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="E4" t="inlineStr">
         <ns0:is>
-          <ns0:t>Shell Companies</ns0:t>
+          <ns0:t>Oil &amp; Gas E&amp;P</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F4" t="inlineStr">
         <ns0:is>
-          <ns0:t>주요 영업활동 없이 기업과의 합병, 주식 교환, 자산 인수 등 사업결합을 추진.</ns0:t>
+          <ns0:t>미국·이집트·북해에서 천연가스·원유·천연가스액을 탐사·개발·생산하는 독립 에너지 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G4">
-        <ns0:v>10.979999542236328</ns0:v>
+        <ns0:v>47.369998931884766</ns0:v>
       </ns0:c>
       <ns0:c r="H4">
-        <ns0:v>1.4787416998601755</ns0:v>
+        <ns0:v>-1.3330543887175805</ns0:v>
       </ns0:c>
       <ns0:c r="I4">
-        <ns0:v>10.859999656677246</ns0:v>
+        <ns0:v>48.08000183105469</ns0:v>
       </ns0:c>
       <ns0:c r="J4">
-        <ns0:v>1.1049713568388686</ns0:v>
+        <ns0:v>-1.4767114644977708</ns0:v>
+      </ns0:c>
+      <ns0:c r="K4">
+        <ns0:v>0.8837884965251704</ns0:v>
       </ns0:c>
       <ns0:c r="L4">
-        <ns0:v>94.11871785465019</ns0:v>
+        <ns0:v>64.69187965552572</ns0:v>
       </ns0:c>
       <ns0:c r="M4">
-        <ns0:v>10.829999732971192</ns0:v>
+        <ns0:v>44.24850006103516</ns0:v>
       </ns0:c>
       <ns0:c r="N4">
-        <ns0:v>10.801599884033203</ns0:v>
+        <ns0:v>43.109000015258786</ns0:v>
       </ns0:c>
       <ns0:c r="O4">
-        <ns0:v>10.65395495414734</ns0:v>
+        <ns0:v>36.19505007743835</ns0:v>
       </ns0:c>
       <ns0:c r="P4" t="inlineStr">
         <ns0:is>
-          <ns0:t>종가 돌파</ns0:t>
+          <ns0:t>장중 경신 후 밀림</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="Q4" t="inlineStr">
@@ -344,7 +344,7 @@
       </ns0:c>
       <ns0:c r="T4" t="inlineStr">
         <ns0:is>
-          <ns0:t>https://finance.yahoo.com/quote/ALDF/profile/</ns0:t>
+          <ns0:t>https://finance.yahoo.com/quote/APA/profile/</ns0:t>
         </ns0:is>
       </ns0:c>
     </ns0:row>
@@ -356,55 +356,55 @@
       </ns0:c>
       <ns0:c r="B5" t="inlineStr">
         <ns0:is>
-          <ns0:t>APA</ns0:t>
+          <ns0:t>ASC</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="C5" t="inlineStr">
         <ns0:is>
-          <ns0:t>APA Corp</ns0:t>
+          <ns0:t>Ardmore Shipping Corp</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D5" t="inlineStr">
         <ns0:is>
-          <ns0:t>Energy</ns0:t>
+          <ns0:t>Industrials</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="E5" t="inlineStr">
         <ns0:is>
-          <ns0:t>Oil &amp; Gas E&amp;P</ns0:t>
+          <ns0:t>Marine Shipping</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F5" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국·이집트·북해에서 천연가스, 원유 및 천연가스액을 탐사·개발·생산하는 독립 에너지 기업.</ns0:t>
+          <ns0:t>전 세계에서 석유제품과 화학제품을 해상 운송하는 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G5">
-        <ns0:v>47.369998931884766</ns0:v>
+        <ns0:v>19.670000076293945</ns0:v>
       </ns0:c>
       <ns0:c r="H5">
-        <ns0:v>-1.3330543887175805</ns0:v>
+        <ns0:v>-2.2851420946365275</ns0:v>
       </ns0:c>
       <ns0:c r="I5">
-        <ns0:v>48.08000183105469</ns0:v>
+        <ns0:v>20.149999618530273</ns0:v>
       </ns0:c>
       <ns0:c r="J5">
-        <ns0:v>-1.4767114644977708</ns0:v>
+        <ns0:v>-2.382131768354534</ns0:v>
       </ns0:c>
       <ns0:c r="K5">
-        <ns0:v>0.8837884965251704</ns0:v>
+        <ns0:v>1.3509094790462801</ns0:v>
       </ns0:c>
       <ns0:c r="L5">
-        <ns0:v>64.69187965552572</ns0:v>
+        <ns0:v>59.93280844247997</ns0:v>
       </ns0:c>
       <ns0:c r="M5">
-        <ns0:v>44.24850006103516</ns0:v>
+        <ns0:v>18.82599992752075</ns0:v>
       </ns0:c>
       <ns0:c r="N5">
-        <ns0:v>43.109000015258786</ns0:v>
+        <ns0:v>18.188199882507323</ns0:v>
       </ns0:c>
       <ns0:c r="O5">
-        <ns0:v>36.19505007743835</ns0:v>
+        <ns0:v>16.08799996852875</ns0:v>
       </ns0:c>
       <ns0:c r="P5" t="inlineStr">
         <ns0:is>
@@ -423,7 +423,7 @@
       </ns0:c>
       <ns0:c r="T5" t="inlineStr">
         <ns0:is>
-          <ns0:t>https://finance.yahoo.com/quote/APA/profile/</ns0:t>
+          <ns0:t>https://finance.yahoo.com/quote/ASC/profile/</ns0:t>
         </ns0:is>
       </ns0:c>
     </ns0:row>
@@ -435,12 +435,12 @@
       </ns0:c>
       <ns0:c r="B6" t="inlineStr">
         <ns0:is>
-          <ns0:t>ASC</ns0:t>
+          <ns0:t>ATKR</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="C6" t="inlineStr">
         <ns0:is>
-          <ns0:t>Ardmore Shipping Corp</ns0:t>
+          <ns0:t>Atkore Inc</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D6" t="inlineStr">
@@ -450,44 +450,44 @@
       </ns0:c>
       <ns0:c r="E6" t="inlineStr">
         <ns0:is>
-          <ns0:t>Marine Shipping</ns0:t>
+          <ns0:t>Electrical Equipment &amp; Parts</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F6" t="inlineStr">
         <ns0:is>
-          <ns0:t>전 세계에서 석유제품과 화학제품을 해상 운송하는 기업.</ns0:t>
+          <ns0:t>전기·기계·안전·인프라 제품과 솔루션을 제조·판매하는 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G6">
-        <ns0:v>19.670000076293945</ns0:v>
+        <ns0:v>94.93000030517578</ns0:v>
       </ns0:c>
       <ns0:c r="H6">
-        <ns0:v>-2.2851420946365275</ns0:v>
+        <ns0:v>0.052701362990403844</ns0:v>
       </ns0:c>
       <ns0:c r="I6">
-        <ns0:v>20.149999618530273</ns0:v>
+        <ns0:v>94.9000015258789</ns0:v>
       </ns0:c>
       <ns0:c r="J6">
-        <ns0:v>-2.382131768354534</ns0:v>
+        <ns0:v>0.0316109365801065</ns0:v>
       </ns0:c>
       <ns0:c r="K6">
-        <ns0:v>1.3509094790462801</ns0:v>
+        <ns0:v>1.149775972643658</ns0:v>
       </ns0:c>
       <ns0:c r="L6">
-        <ns0:v>59.93280844247997</ns0:v>
+        <ns0:v>72.23885089238354</ns0:v>
       </ns0:c>
       <ns0:c r="M6">
-        <ns0:v>18.82599992752075</ns0:v>
+        <ns0:v>94.67849960327149</ns0:v>
       </ns0:c>
       <ns0:c r="N6">
-        <ns0:v>18.188199882507323</ns0:v>
+        <ns0:v>94.14320022583007</ns0:v>
       </ns0:c>
       <ns0:c r="O6">
-        <ns0:v>16.08799996852875</ns0:v>
+        <ns0:v>76.60020009994507</ns0:v>
       </ns0:c>
       <ns0:c r="P6" t="inlineStr">
         <ns0:is>
-          <ns0:t>장중 경신 후 밀림</ns0:t>
+          <ns0:t>종가 돌파</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="Q6" t="inlineStr">
@@ -502,7 +502,7 @@
       </ns0:c>
       <ns0:c r="T6" t="inlineStr">
         <ns0:is>
-          <ns0:t>https://finance.yahoo.com/quote/ASC/profile/</ns0:t>
+          <ns0:t>https://finance.yahoo.com/quote/ATKR/profile/</ns0:t>
         </ns0:is>
       </ns0:c>
     </ns0:row>
@@ -534,7 +534,7 @@
       </ns0:c>
       <ns0:c r="F7" t="inlineStr">
         <ns0:is>
-          <ns0:t>다양한 규모의 조직이 장소와 기기에 관계없이 콘텐츠를 관리하는 클라우드 플랫폼 제공.</ns0:t>
+          <ns0:t>다양한 규모의 조직이 장소·기기에 관계없이 콘텐츠를 관리하는 클라우드 플랫폼 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G7">
@@ -613,7 +613,7 @@
       </ns0:c>
       <ns0:c r="F8" t="inlineStr">
         <ns0:is>
-          <ns0:t>전 세계에서 석유·가스 사업을 운영하며 가스·저탄소 에너지, 석유 생산 및 고객·제품 부문을 영위.</ns0:t>
+          <ns0:t>전 세계에서 가스·저탄소 에너지, 석유 생산, 고객·제품 부문 등 석유·가스 사업 운영.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G8">
@@ -692,7 +692,7 @@
       </ns0:c>
       <ns0:c r="F9" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국 의료기술 기업으로 급성기 환자용 현장 뇌파검사 플랫폼인 Ceribell System을 개발.</ns0:t>
+          <ns0:t>급성기 환자용 현장 뇌파검사 플랫폼 Ceribell System을 개발하는 미국 의료기술 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G9">
@@ -850,7 +850,7 @@
       </ns0:c>
       <ns0:c r="F11" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국과 싱가포르에서 광고판·포스터 등을 활용한 옥외 및 공항 광고 서비스를 제공하는 기업.</ns0:t>
+          <ns0:t>미국·싱가포르에서 광고판·포스터 등을 활용한 옥외·공항 광고 서비스를 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G11">
@@ -929,7 +929,7 @@
       </ns0:c>
       <ns0:c r="F12" t="inlineStr">
         <ns0:is>
-          <ns0:t>대만과 해외에서 개인·기업 고객에게 이동통신·유선통신 등 통합 통신 서비스를 제공하는 기업.</ns0:t>
+          <ns0:t>대만과 해외 개인·기업 고객에게 이동통신·유선통신 등 통합 통신 서비스를 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G12">
@@ -1008,7 +1008,7 @@
       </ns0:c>
       <ns0:c r="F13" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국에서 보험 보장이 부족한 가정과 기업에 프로그램·서비스를 제공하는 관리형 의료 기업.</ns0:t>
+          <ns0:t>미국 내 보험 보장이 부족한 가정·기업에 프로그램과 서비스를 제공하는 관리형 의료 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G13">
@@ -1087,7 +1087,7 @@
       </ns0:c>
       <ns0:c r="F14" t="inlineStr">
         <ns0:is>
-          <ns0:t>캐나다 서부·영국 북해·아프리카 해상에서 원유·천연가스·천연가스액을 탐사·개발·생산·판매하는 기업.</ns0:t>
+          <ns0:t>캐나다 서부·영국 북해·아프리카 해상에서 원유·천연가스·천연가스액을 탐사·개발·생산·판매.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G14">
@@ -1166,7 +1166,7 @@
       </ns0:c>
       <ns0:c r="F15" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국에서 직업건강센터와 사업장 내 진료소 등을 통해 직업건강 및 고용주·소비자 건강 서비스를 제공.</ns0:t>
+          <ns0:t>미국에서 직업건강센터와 사업장 내 진료소를 통해 직업건강 및 고용주·소비자 건강 서비스를 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G15">
@@ -1245,7 +1245,7 @@
       </ns0:c>
       <ns0:c r="F16" t="inlineStr">
         <ns0:is>
-          <ns0:t>원유·역청·천연가스·액화천연가스·천연가스액을 탐사·생산·운송·판매하는 기업.</ns0:t>
+          <ns0:t>원유·역청·천연가스·액화천연가스·천연가스액을 탐사·생산·운송·판매.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G16">
@@ -1324,7 +1324,7 @@
       </ns0:c>
       <ns0:c r="F17" t="inlineStr">
         <ns0:is>
-          <ns0:t>AI 등 기술을 활용해 산재보상·일반 및 자동차 배상책임 관리와 병원비 심사·지급 적정성 솔루션을 제공.</ns0:t>
+          <ns0:t>AI 등을 활용해 산재보상·일반 및 자동차 배상책임 관리, 병원비 심사·지급 적정성 솔루션을 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G17">
@@ -1403,7 +1403,7 @@
       </ns0:c>
       <ns0:c r="F18" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국에서 재생연료, 석유 정제·판매 및 질소비료 제조 사업을 영위하는 기업.</ns0:t>
+          <ns0:t>미국에서 재생연료, 석유 정제·판매, 질소비료 제조 사업을 운영.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G18">
@@ -1482,7 +1482,7 @@
       </ns0:c>
       <ns0:c r="F19" t="inlineStr">
         <ns0:is>
-          <ns0:t>원유·천연가스 탐사, 개발, 생산, 운송 등을 포함한 통합 에너지 및 화학 사업을 영위.</ns0:t>
+          <ns0:t>원유·천연가스 탐사·개발·생산·운송 등을 포함한 통합 에너지·화학 사업 영위.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G19">
@@ -1561,7 +1561,7 @@
       </ns0:c>
       <ns0:c r="F20" t="inlineStr">
         <ns0:is>
-          <ns0:t>중국에서 학습 서비스·스마트 기기·온라인 마케팅을 비롯한 인터넷 서비스를 제공하는 기업.</ns0:t>
+          <ns0:t>중국에서 학습 서비스·스마트 기기·온라인 마케팅 등 인터넷 서비스를 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G20">
@@ -1640,7 +1640,7 @@
       </ns0:c>
       <ns0:c r="F21" t="inlineStr">
         <ns0:is>
-          <ns0:t>자회사를 통해 원유 운반선을 소유·운영하며 기술 관리 서비스도 제공하는 기업.</ns0:t>
+          <ns0:t>자회사를 통해 원유 운반선을 소유·운영하고 기술 관리 서비스 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G21">
@@ -1719,7 +1719,7 @@
       </ns0:c>
       <ns0:c r="F22" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국 독립 에너지 기업으로 정유·재생에너지·마케팅·윤활유·미드스트림 사업과 연료 생산·판매를 수행.</ns0:t>
+          <ns0:t>미국 독립 에너지 기업으로 정유·재생에너지·윤활유·미드스트림 사업과 연료 생산·판매 수행.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G22">
@@ -1877,7 +1877,7 @@
       </ns0:c>
       <ns0:c r="F24" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국·트리니다드토바고 등에서 원유·천연가스액·천연가스를 탐사·개발·생산·판매하는 기업.</ns0:t>
+          <ns0:t>미국·트리니다드토바고 등에서 원유·천연가스액·천연가스를 탐사·개발·생산·판매.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G24">
@@ -2035,7 +2035,7 @@
       </ns0:c>
       <ns0:c r="F26" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국·호주·유럽의 매장과 온라인에서 게임, 수집품, 엔터테인먼트 제품을 판매하는 기업.</ns0:t>
+          <ns0:t>미국·호주·유럽의 매장과 온라인에서 게임·수집품·엔터테인먼트 제품을 판매.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G26">
@@ -2114,7 +2114,7 @@
       </ns0:c>
       <ns0:c r="F27" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국 및 해외에서 에너지 서비스를 제공하며 전력·천연가스 재판매와 재생에너지 사업을 영위.</ns0:t>
+          <ns0:t>미국 및 해외에서 전력·천연가스 재판매와 재생에너지 등 에너지 서비스 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G27">
@@ -2193,7 +2193,7 @@
       </ns0:c>
       <ns0:c r="F28" t="inlineStr">
         <ns0:is>
-          <ns0:t>독자 효소와 기기를 연구·개발·상용화하며 재조합 인간 히알루로니다아제 기반 제품을 보유한 바이오제약사.</ns0:t>
+          <ns0:t>독자 효소·기기를 연구·개발·상용화하며 재조합 인간 히알루로니다아제 기반 제품을 보유한 바이오제약사.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G28">
@@ -2272,7 +2272,7 @@
       </ns0:c>
       <ns0:c r="F29" t="inlineStr">
         <ns0:is>
-          <ns0:t>중국과 해외에서 다양한 형태의 맞춤형 냉간 성형 강재를 제조·판매하는 회사.</ns0:t>
+          <ns0:t>중국과 해외에서 다양한 맞춤형 냉간 성형 강재를 제조·판매한다.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G29">
@@ -2351,7 +2351,7 @@
       </ns0:c>
       <ns0:c r="F30" t="inlineStr">
         <ns0:is>
-          <ns0:t>세계 각지에서 오토바이·자동차·동력 제품을 개발·제조·유통하고 금융 서비스를 제공하는 기업.</ns0:t>
+          <ns0:t>세계 각지에서 오토바이·자동차·동력 제품을 개발·제조·유통하고 금융 서비스를 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G30">
@@ -2430,7 +2430,7 @@
       </ns0:c>
       <ns0:c r="F31" t="inlineStr">
         <ns0:is>
-          <ns0:t>기술 기반 고객 경험 솔루션과 고객서비스·기술지원·백오피스 아웃소싱을 제공하는 기업.</ns0:t>
+          <ns0:t>기술 기반 고객 경험 솔루션과 고객서비스·기술지원·백오피스 아웃소싱을 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G31">
@@ -2509,7 +2509,7 @@
       </ns0:c>
       <ns0:c r="F32" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국 소비재 브랜드 등의 디지털 판촉을 제휴 매체 네트워크를 통해 소비자에게 제공.</ns0:t>
+          <ns0:t>미국 소비재 브랜드 등의 디지털 판촉을 제휴 매체 네트워크로 소비자에게 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G32">
@@ -2588,7 +2588,7 @@
       </ns0:c>
       <ns0:c r="F33" t="inlineStr">
         <ns0:is>
-          <ns0:t>식품·음료·건강 및 바이오과학·향료와 관련 제품을 제조·판매하는 글로벌 기업.</ns0:t>
+          <ns0:t>식품·음료·건강·바이오과학·향료 관련 제품을 제조·판매하는 글로벌 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G33">
@@ -2667,7 +2667,7 @@
       </ns0:c>
       <ns0:c r="F34" t="inlineStr">
         <ns0:is>
-          <ns0:t>원유와 석유제품의 국제 해상 운송을 위해 원유선과 제품 운반선을 보유·운영하는 기업.</ns0:t>
+          <ns0:t>원유선과 석유제품 운반선을 보유·운영하며 원유·석유제품의 국제 해상 운송을 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G34">
@@ -2746,7 +2746,7 @@
       </ns0:c>
       <ns0:c r="F35" t="inlineStr">
         <ns0:is>
-          <ns0:t>중국에서 푸시 알림·메신저·분석·문자·원클릭 인증 등 개발자 서비스와 산업별 앱을 제공하는 기업.</ns0:t>
+          <ns0:t>중국에서 푸시 알림·메신저·분석·문자·원클릭 인증 등 개발자 서비스와 산업별 앱을 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G35">
@@ -2825,7 +2825,7 @@
       </ns0:c>
       <ns0:c r="F36" t="inlineStr">
         <ns0:is>
-          <ns0:t>소셜 서비스와 통신 기술을 제공하며 소셜 라이브 스트리밍 플랫폼 Bigo Live를 운영한다.</ns0:t>
+          <ns0:t>소셜 서비스·통신 기술을 제공하고 소셜 라이브 스트리밍 플랫폼 Bigo Live를 운영.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G36">
@@ -3062,7 +3062,7 @@
       </ns0:c>
       <ns0:c r="F39" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국 석유·천연가스 자산의 광물권과 로열티 권익을 보유·취득하는 기업.</ns0:t>
+          <ns0:t>미국 석유·천연가스 자산의 광물권과 로열티 권익을 보유·취득.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G39">
@@ -3141,7 +3141,7 @@
       </ns0:c>
       <ns0:c r="F40" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국과 해외에서 거래 처리 및 결제 관련 제품·서비스를 소비자, 가맹점, 금융기관 등에 제공.</ns0:t>
+          <ns0:t>미국과 해외에서 소비자·가맹점·금융기관 등에 거래 처리와 결제 제품·서비스를 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G40">
@@ -3220,7 +3220,7 @@
       </ns0:c>
       <ns0:c r="F41" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국의 통합 다운스트림 에너지 기업으로 정유·판매, 미드스트림, 재생 디젤 사업을 운영한다.</ns0:t>
+          <ns0:t>미국에서 정유·판매, 미드스트림, 재생 디젤 사업을 운영하는 통합 다운스트림 에너지 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G41">
@@ -3299,7 +3299,7 @@
       </ns0:c>
       <ns0:c r="F42" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국·캐나다·멕시코·영국 등에서 금속가공 및 유지보수·수리·운영용 제품과 서비스를 유통한다.</ns0:t>
+          <ns0:t>미국·캐나다·멕시코·영국 등에서 금속가공 및 유지보수·수리·운영용 제품과 서비스를 유통.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G42">
@@ -3378,7 +3378,7 @@
       </ns0:c>
       <ns0:c r="F43" t="inlineStr">
         <ns0:is>
-          <ns0:t>전 세계에 실험실용 기기 등 정밀기기를 제조·공급하고 관련 서비스를 제공한다.</ns0:t>
+          <ns0:t>전 세계에 실험실용 기기 등 정밀기기를 제조·공급하고 관련 서비스 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G43">
@@ -3457,7 +3457,7 @@
       </ns0:c>
       <ns0:c r="F44" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국에서 식음료 판매, 컨설팅, 전자폐기물 자재 판매 등 공급망 사업을 운영한다.</ns0:t>
+          <ns0:t>미국에서 식음료 판매, 컨설팅, 전자폐기물 자재 판매 등 공급망 사업을 운영.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G44">
@@ -3536,7 +3536,7 @@
       </ns0:c>
       <ns0:c r="F45" t="inlineStr">
         <ns0:is>
-          <ns0:t>자동차 금융·리스, 은행 및 금융서비스 산업용 기업 소프트웨어를 설계·개발·판매하는 회사.</ns0:t>
+          <ns0:t>자동차 금융·리스, 은행·금융서비스용 기업 소프트웨어를 설계·개발·판매하는 회사.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G45">
@@ -3691,7 +3691,7 @@
       </ns0:c>
       <ns0:c r="F47" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국에서 재생·기존 연료를 공급하며 정유, 소매, 물류 사업을 운영한다.</ns0:t>
+          <ns0:t>미국에서 재생·기존 연료를 공급하며 정유·소매·물류 사업을 운영한다.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G47">
@@ -3770,7 +3770,7 @@
       </ns0:c>
       <ns0:c r="F48" t="inlineStr">
         <ns0:is>
-          <ns0:t>정유·물류 사업을 통해 휘발유·경유·항공유·윤활유·석유화학제품·아스팔트 등을 생산·공급하는 기업.</ns0:t>
+          <ns0:t>정유·물류 사업을 통해 휘발유·경유·항공유·윤활유·석유화학제품·아스팔트를 생산·공급한다.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G48">
@@ -3849,7 +3849,7 @@
       </ns0:c>
       <ns0:c r="F49" t="inlineStr">
         <ns0:is>
-          <ns0:t>브라질과 해외에서 석유·가스를 탐사·생산·판매하며 정유·운송·판매 사업을 운영한다.</ns0:t>
+          <ns0:t>브라질과 해외에서 석유·가스 탐사·생산·판매 및 정유·운송 사업을 운영한다.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G49">
@@ -3928,7 +3928,7 @@
       </ns0:c>
       <ns0:c r="F50" t="inlineStr">
         <ns0:is>
-          <ns0:t>브라질과 해외에서 석유·가스를 탐사·생산·판매하며 정유·운송·판매 사업을 운영한다.</ns0:t>
+          <ns0:t>브라질과 해외에서 석유·가스 탐사·생산·판매 및 정유·운송 사업을 운영한다.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G50">
@@ -4007,7 +4007,7 @@
       </ns0:c>
       <ns0:c r="F51" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국 의료진 대상 비마약성 통증관리·재생건강 솔루션을 개발·제조·판매하며 수술 후 통증관리 주사제를 제공.</ns0:t>
+          <ns0:t>비마약성 통증관리·재생건강 솔루션과 수술 후 통증관리 주사제를 개발·제조·판매.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G51">
@@ -4086,7 +4086,7 @@
       </ns0:c>
       <ns0:c r="F52" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국과 해외에서 바이오의약품을 발굴·개발·제조·마케팅·유통·판매하는 기업.</ns0:t>
+          <ns0:t>미국과 해외에서 바이오의약품을 발굴·개발·제조·마케팅·유통·판매.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G52">
@@ -4165,7 +4165,7 @@
       </ns0:c>
       <ns0:c r="F53" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국 등에서 미드스트림·화학·정유·마케팅 및 특수제품·재생연료 사업을 운영하는 통합 다운스트림 에너지 기업.</ns0:t>
+          <ns0:t>미국 등에서 미드스트림·화학·정유·마케팅·특수제품·재생연료 사업을 운영하는 에너지 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G53">
@@ -4244,7 +4244,7 @@
       </ns0:c>
       <ns0:c r="F54" t="inlineStr">
         <ns0:is>
-          <ns0:t>텍사스·뉴멕시코에서 석유·천연가스·천연가스액 자산을 인수·탐사·개발·생산.</ns0:t>
+          <ns0:t>텍사스·뉴멕시코에서 석유·천연가스·천연가스액 자산을 인수·탐사·개발·생산한다.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G54">
@@ -4323,7 +4323,7 @@
       </ns0:c>
       <ns0:c r="F55" t="inlineStr">
         <ns0:is>
-          <ns0:t>전 세계에서 생명·건강 및 자산집약형 재보험을 제공하며 장애·장기요양 관련 보장도 취급.</ns0:t>
+          <ns0:t>전 세계에서 생명·건강·자산집약형 재보험을 제공하고 장애·장기요양 관련 보장도 취급.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G55">
@@ -4402,7 +4402,7 @@
       </ns0:c>
       <ns0:c r="F56" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국과 해외에서 재산·상해·특종 보험과 재보험을 제공하며 재산 재해 초과손해 재보험을 취급.</ns0:t>
+          <ns0:t>미국과 해외에서 재산·상해·특종 보험 및 재보험을 제공하고 재산 재해 초과손해 재보험 취급.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G56">
@@ -4481,7 +4481,7 @@
       </ns0:c>
       <ns0:c r="F57" t="inlineStr">
         <ns0:is>
-          <ns0:t>세계 각지에서 통합 가스, 자원 개발·생산, 마케팅, 화학·제품, 재생에너지 사업을 운영한다.</ns0:t>
+          <ns0:t>전 세계에서 통합 가스, 자원 개발·생산, 마케팅, 화학·제품, 재생에너지 사업을 운영한다.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G57">
@@ -4560,7 +4560,7 @@
       </ns0:c>
       <ns0:c r="F58" t="inlineStr">
         <ns0:is>
-          <ns0:t>캐나다·미국 등에서 오일샌드, 석유 탐사·생산, 정유·판매 사업을 영위하는 종합 에너지 기업.</ns0:t>
+          <ns0:t>캐나다·미국 등에서 오일샌드, 석유 탐사·생산, 정유·판매 사업을 운영하는 종합 에너지 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G58">
@@ -4639,7 +4639,7 @@
       </ns0:c>
       <ns0:c r="F59" t="inlineStr">
         <ns0:is>
-          <ns0:t>그리스와 해외에서 원유·석유제품 해상 운송 서비스를 제공하며 다양한 유조선과 LNG 운반선 등을 운영.</ns0:t>
+          <ns0:t>그리스와 해외에서 원유·석유제품 해상운송을 제공하며 다양한 유조선과 LNG 운반선 등을 운영.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G59">
@@ -4797,7 +4797,7 @@
       </ns0:c>
       <ns0:c r="F61" t="inlineStr">
         <ns0:is>
-          <ns0:t>버지니아 내 상업·개인 금융 서비스를 제공하는 은행의 지주회사로 은행 및 신탁·상속재산 서비스 운영.</ns0:t>
+          <ns0:t>버지니아에서 상업·개인 금융과 신탁·상속재산 서비스를 운영하는 은행 지주회사.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G61">
@@ -4876,7 +4876,7 @@
       </ns0:c>
       <ns0:c r="F62" t="inlineStr">
         <ns0:is>
-          <ns0:t>주식·뮤추얼펀드·ETF·옵션 등을 다루는 투자 정기간행물과 관련 출판물을 제작·판매.</ns0:t>
+          <ns0:t>주식·뮤추얼펀드·ETF·옵션 관련 투자 정기간행물과 출판물을 제작·판매하는 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G62">
@@ -4955,7 +4955,7 @@
       </ns0:c>
       <ns0:c r="F63" t="inlineStr">
         <ns0:is>
-          <ns0:t>석유 기반·저탄소 운송용 액체 연료와 석유화학 제품을 제조·판매하는 기업.</ns0:t>
+          <ns0:t>석유 기반·저탄소 운송용 액체 연료와 석유화학 제품을 제조·판매한다.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G63">
@@ -5113,7 +5113,7 @@
       </ns0:c>
       <ns0:c r="F65" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국·캐나다 등에서 원유·천연가스를 탐사·생산하며 에너지·화학·특수제품 사업을 운영한다.</ns0:t>
+          <ns0:t>미국·캐나다 등에서 원유·천연가스를 탐사·생산하며 에너지·화학·특수제품 사업 운영.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G65">

</xml_diff>